<commit_message>
Add monster CSV table, fix EXP progression, and circular minimap.
Wire monster stats from CSV on spawn with mon_type for normal/boss rules.
Use per-level exp from player_stats_default.csv instead of cumulative values.
Merge circular minimap layout into RadarMinimapView and fix HUD prefab references.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/테이블/player_stats_default.xlsx
+++ b/테이블/player_stats_default.xlsx
@@ -49,10 +49,6 @@
     <t>level</t>
   </si>
   <si>
-    <t>exp</t>
-    <phoneticPr fontId="18" type="noConversion"/>
-  </si>
-  <si>
     <t>stat_id</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
@@ -62,6 +58,10 @@
   </si>
   <si>
     <t>mp</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>need_exp</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -1012,19 +1012,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -1035,7 +1035,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="D2" s="1">
         <v>10</v>
@@ -1052,7 +1052,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="1">
-        <v>500</v>
+        <v>800</v>
       </c>
       <c r="D3" s="1">
         <v>15</v>
@@ -1069,7 +1069,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="1">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="D4" s="1">
         <v>20</v>
@@ -1086,7 +1086,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="1">
-        <v>1500</v>
+        <v>1400</v>
       </c>
       <c r="D5" s="1">
         <v>25</v>
@@ -1103,7 +1103,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="1">
-        <v>2000</v>
+        <v>1700</v>
       </c>
       <c r="D6" s="1">
         <v>30</v>
@@ -1120,7 +1120,7 @@
         <v>6</v>
       </c>
       <c r="C7" s="1">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="D7" s="1">
         <v>35</v>
@@ -1137,7 +1137,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="1">
-        <v>3000</v>
+        <v>2300</v>
       </c>
       <c r="D8" s="1">
         <v>40</v>
@@ -1154,7 +1154,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="1">
-        <v>3500</v>
+        <v>2600</v>
       </c>
       <c r="D9" s="1">
         <v>45</v>
@@ -1171,7 +1171,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="1">
-        <v>4000</v>
+        <v>2900</v>
       </c>
       <c r="D10" s="1">
         <v>50</v>
@@ -1188,7 +1188,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="1">
-        <v>4500</v>
+        <v>3200</v>
       </c>
       <c r="D11" s="1">
         <v>55</v>
@@ -1205,7 +1205,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="1">
-        <v>5500</v>
+        <v>3600</v>
       </c>
       <c r="D12" s="1">
         <v>60</v>
@@ -1222,7 +1222,7 @@
         <v>12</v>
       </c>
       <c r="C13" s="1">
-        <v>6500</v>
+        <v>4000</v>
       </c>
       <c r="D13" s="1">
         <v>65</v>
@@ -1239,7 +1239,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="1">
-        <v>7500</v>
+        <v>4400</v>
       </c>
       <c r="D14" s="1">
         <v>70</v>
@@ -1256,7 +1256,7 @@
         <v>14</v>
       </c>
       <c r="C15" s="1">
-        <v>8500</v>
+        <v>4800</v>
       </c>
       <c r="D15" s="1">
         <v>75</v>
@@ -1273,7 +1273,7 @@
         <v>15</v>
       </c>
       <c r="C16" s="1">
-        <v>9500</v>
+        <v>5200</v>
       </c>
       <c r="D16" s="1">
         <v>80</v>
@@ -1290,7 +1290,7 @@
         <v>16</v>
       </c>
       <c r="C17" s="1">
-        <v>10500</v>
+        <v>5600</v>
       </c>
       <c r="D17" s="1">
         <v>85</v>
@@ -1307,7 +1307,7 @@
         <v>17</v>
       </c>
       <c r="C18" s="1">
-        <v>11500</v>
+        <v>6000</v>
       </c>
       <c r="D18" s="1">
         <v>90</v>
@@ -1324,7 +1324,7 @@
         <v>18</v>
       </c>
       <c r="C19" s="1">
-        <v>12500</v>
+        <v>6400</v>
       </c>
       <c r="D19" s="1">
         <v>95</v>
@@ -1341,7 +1341,7 @@
         <v>19</v>
       </c>
       <c r="C20" s="1">
-        <v>13500</v>
+        <v>6800</v>
       </c>
       <c r="D20" s="1">
         <v>100</v>
@@ -1358,7 +1358,7 @@
         <v>20</v>
       </c>
       <c r="C21" s="1">
-        <v>14500</v>
+        <v>7200</v>
       </c>
       <c r="D21" s="1">
         <v>105</v>
@@ -1375,7 +1375,7 @@
         <v>21</v>
       </c>
       <c r="C22" s="1">
-        <v>16000</v>
+        <v>7700</v>
       </c>
       <c r="D22" s="1">
         <v>110</v>
@@ -1392,7 +1392,7 @@
         <v>22</v>
       </c>
       <c r="C23" s="1">
-        <v>17500</v>
+        <v>8200</v>
       </c>
       <c r="D23" s="1">
         <v>115</v>
@@ -1409,7 +1409,7 @@
         <v>23</v>
       </c>
       <c r="C24" s="1">
-        <v>19000</v>
+        <v>8700</v>
       </c>
       <c r="D24" s="1">
         <v>120</v>
@@ -1426,7 +1426,7 @@
         <v>24</v>
       </c>
       <c r="C25" s="1">
-        <v>20500</v>
+        <v>9200</v>
       </c>
       <c r="D25" s="1">
         <v>125</v>
@@ -1443,7 +1443,7 @@
         <v>25</v>
       </c>
       <c r="C26" s="1">
-        <v>22000</v>
+        <v>9700</v>
       </c>
       <c r="D26" s="1">
         <v>130</v>
@@ -1460,7 +1460,7 @@
         <v>26</v>
       </c>
       <c r="C27" s="1">
-        <v>23500</v>
+        <v>10200</v>
       </c>
       <c r="D27" s="1">
         <v>135</v>
@@ -1477,7 +1477,7 @@
         <v>27</v>
       </c>
       <c r="C28" s="1">
-        <v>25000</v>
+        <v>10700</v>
       </c>
       <c r="D28" s="1">
         <v>140</v>
@@ -1494,7 +1494,7 @@
         <v>28</v>
       </c>
       <c r="C29" s="1">
-        <v>26500</v>
+        <v>11200</v>
       </c>
       <c r="D29" s="1">
         <v>145</v>
@@ -1511,7 +1511,7 @@
         <v>29</v>
       </c>
       <c r="C30" s="1">
-        <v>28000</v>
+        <v>11700</v>
       </c>
       <c r="D30" s="1">
         <v>150</v>
@@ -1528,7 +1528,7 @@
         <v>30</v>
       </c>
       <c r="C31" s="1">
-        <v>29500</v>
+        <v>12200</v>
       </c>
       <c r="D31" s="1">
         <v>155</v>
@@ -1545,7 +1545,7 @@
         <v>31</v>
       </c>
       <c r="C32" s="1">
-        <v>31500</v>
+        <v>12800</v>
       </c>
       <c r="D32" s="1">
         <v>160</v>
@@ -1562,7 +1562,7 @@
         <v>32</v>
       </c>
       <c r="C33" s="1">
-        <v>33500</v>
+        <v>13400</v>
       </c>
       <c r="D33" s="1">
         <v>165</v>
@@ -1579,7 +1579,7 @@
         <v>33</v>
       </c>
       <c r="C34" s="1">
-        <v>35500</v>
+        <v>14000</v>
       </c>
       <c r="D34" s="1">
         <v>170</v>
@@ -1596,7 +1596,7 @@
         <v>34</v>
       </c>
       <c r="C35" s="1">
-        <v>37500</v>
+        <v>14600</v>
       </c>
       <c r="D35" s="1">
         <v>175</v>
@@ -1613,7 +1613,7 @@
         <v>35</v>
       </c>
       <c r="C36" s="1">
-        <v>39500</v>
+        <v>15200</v>
       </c>
       <c r="D36" s="1">
         <v>180</v>
@@ -1630,7 +1630,7 @@
         <v>36</v>
       </c>
       <c r="C37" s="1">
-        <v>41500</v>
+        <v>15800</v>
       </c>
       <c r="D37" s="1">
         <v>185</v>
@@ -1647,7 +1647,7 @@
         <v>37</v>
       </c>
       <c r="C38" s="1">
-        <v>43500</v>
+        <v>16400</v>
       </c>
       <c r="D38" s="1">
         <v>190</v>
@@ -1664,7 +1664,7 @@
         <v>38</v>
       </c>
       <c r="C39" s="1">
-        <v>45500</v>
+        <v>17000</v>
       </c>
       <c r="D39" s="1">
         <v>195</v>
@@ -1681,7 +1681,7 @@
         <v>39</v>
       </c>
       <c r="C40" s="1">
-        <v>47500</v>
+        <v>17600</v>
       </c>
       <c r="D40" s="1">
         <v>200</v>
@@ -1698,7 +1698,7 @@
         <v>40</v>
       </c>
       <c r="C41" s="1">
-        <v>49500</v>
+        <v>18200</v>
       </c>
       <c r="D41" s="1">
         <v>205</v>
@@ -1715,7 +1715,7 @@
         <v>41</v>
       </c>
       <c r="C42" s="1">
-        <v>52000</v>
+        <v>18900</v>
       </c>
       <c r="D42" s="1">
         <v>210</v>
@@ -1732,7 +1732,7 @@
         <v>42</v>
       </c>
       <c r="C43" s="1">
-        <v>54500</v>
+        <v>19600</v>
       </c>
       <c r="D43" s="1">
         <v>215</v>
@@ -1749,7 +1749,7 @@
         <v>43</v>
       </c>
       <c r="C44" s="1">
-        <v>57000</v>
+        <v>20300</v>
       </c>
       <c r="D44" s="1">
         <v>220</v>
@@ -1766,7 +1766,7 @@
         <v>44</v>
       </c>
       <c r="C45" s="1">
-        <v>59500</v>
+        <v>21000</v>
       </c>
       <c r="D45" s="1">
         <v>225</v>
@@ -1783,7 +1783,7 @@
         <v>45</v>
       </c>
       <c r="C46" s="1">
-        <v>62000</v>
+        <v>21700</v>
       </c>
       <c r="D46" s="1">
         <v>230</v>
@@ -1800,7 +1800,7 @@
         <v>46</v>
       </c>
       <c r="C47" s="1">
-        <v>64500</v>
+        <v>22400</v>
       </c>
       <c r="D47" s="1">
         <v>235</v>
@@ -1817,7 +1817,7 @@
         <v>47</v>
       </c>
       <c r="C48" s="1">
-        <v>67000</v>
+        <v>23100</v>
       </c>
       <c r="D48" s="1">
         <v>240</v>
@@ -1834,7 +1834,7 @@
         <v>48</v>
       </c>
       <c r="C49" s="1">
-        <v>69500</v>
+        <v>23800</v>
       </c>
       <c r="D49" s="1">
         <v>245</v>
@@ -1851,7 +1851,7 @@
         <v>49</v>
       </c>
       <c r="C50" s="1">
-        <v>72000</v>
+        <v>24500</v>
       </c>
       <c r="D50" s="1">
         <v>250</v>
@@ -1868,7 +1868,7 @@
         <v>50</v>
       </c>
       <c r="C51" s="1">
-        <v>74500</v>
+        <v>25200</v>
       </c>
       <c r="D51" s="1">
         <v>255</v>
@@ -1901,26 +1901,26 @@
       <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B3" s="1">
         <v>1</v>
       </c>
       <c r="C3" s="1">
-        <v>0</v>
-      </c>
-      <c r="F3" s="3" t="s">
+        <v>500</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1930,16 +1930,16 @@
       </c>
       <c r="C4" s="1">
         <f>C3+$H$4</f>
-        <v>500</v>
-      </c>
-      <c r="F4" s="3">
+        <v>800</v>
+      </c>
+      <c r="F4" s="2">
         <v>1</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="2">
         <v>10</v>
       </c>
-      <c r="H4" s="3">
-        <v>500</v>
+      <c r="H4" s="2">
+        <v>300</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.3">
@@ -1947,17 +1947,17 @@
         <v>3</v>
       </c>
       <c r="C5" s="1">
-        <f t="shared" ref="C5:C13" si="0">C4+$H$4</f>
-        <v>1000</v>
-      </c>
-      <c r="F5" s="3">
+        <f t="shared" ref="C5:C12" si="0">C4+$H$4</f>
+        <v>1100</v>
+      </c>
+      <c r="F5" s="2">
         <v>11</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="2">
         <v>20</v>
       </c>
-      <c r="H5" s="3">
-        <v>1000</v>
+      <c r="H5" s="2">
+        <v>400</v>
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.3">
@@ -1966,16 +1966,16 @@
       </c>
       <c r="C6" s="1">
         <f t="shared" si="0"/>
-        <v>1500</v>
-      </c>
-      <c r="F6" s="3">
+        <v>1400</v>
+      </c>
+      <c r="F6" s="2">
         <v>21</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="2">
         <v>30</v>
       </c>
-      <c r="H6" s="3">
-        <v>1500</v>
+      <c r="H6" s="2">
+        <v>500</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.3">
@@ -1984,16 +1984,16 @@
       </c>
       <c r="C7" s="1">
         <f t="shared" si="0"/>
-        <v>2000</v>
-      </c>
-      <c r="F7" s="3">
+        <v>1700</v>
+      </c>
+      <c r="F7" s="2">
         <v>31</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="2">
         <v>40</v>
       </c>
-      <c r="H7" s="3">
-        <v>2000</v>
+      <c r="H7" s="2">
+        <v>600</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.3">
@@ -2002,16 +2002,16 @@
       </c>
       <c r="C8" s="1">
         <f t="shared" si="0"/>
-        <v>2500</v>
-      </c>
-      <c r="F8" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F8" s="2">
         <v>41</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="2">
         <v>50</v>
       </c>
-      <c r="H8" s="3">
-        <v>2500</v>
+      <c r="H8" s="2">
+        <v>700</v>
       </c>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.3">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="C9" s="1">
         <f t="shared" si="0"/>
-        <v>3000</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.3">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="C10" s="1">
         <f t="shared" si="0"/>
-        <v>3500</v>
+        <v>2600</v>
       </c>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.3">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="C11" s="1">
         <f t="shared" si="0"/>
-        <v>4000</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.3">
@@ -2047,7 +2047,7 @@
       </c>
       <c r="C12" s="1">
         <f t="shared" si="0"/>
-        <v>4500</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.3">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="C13" s="1">
         <f>C12+$H$5</f>
-        <v>5500</v>
+        <v>3600</v>
       </c>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.3">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="C14" s="1">
         <f t="shared" ref="C14:C22" si="1">C13+$H$5</f>
-        <v>6500</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.3">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="C15" s="1">
         <f t="shared" si="1"/>
-        <v>7500</v>
+        <v>4400</v>
       </c>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="C16" s="1">
         <f t="shared" si="1"/>
-        <v>8500</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.3">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="C17" s="1">
         <f t="shared" si="1"/>
-        <v>9500</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.3">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="C18" s="1">
         <f t="shared" si="1"/>
-        <v>10500</v>
+        <v>5600</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.3">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="C19" s="1">
         <f t="shared" si="1"/>
-        <v>11500</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.3">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="C20" s="1">
         <f t="shared" si="1"/>
-        <v>12500</v>
+        <v>6400</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.3">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="C21" s="1">
         <f t="shared" si="1"/>
-        <v>13500</v>
+        <v>6800</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.3">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="C22" s="1">
         <f t="shared" si="1"/>
-        <v>14500</v>
+        <v>7200</v>
       </c>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.3">
@@ -2146,7 +2146,7 @@
       </c>
       <c r="C23" s="1">
         <f>C22+$H$6</f>
-        <v>16000</v>
+        <v>7700</v>
       </c>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.3">
@@ -2154,8 +2154,8 @@
         <v>22</v>
       </c>
       <c r="C24" s="1">
-        <f t="shared" ref="C24:C33" si="2">C23+$H$6</f>
-        <v>17500</v>
+        <f t="shared" ref="C24:C32" si="2">C23+$H$6</f>
+        <v>8200</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.3">
@@ -2164,7 +2164,7 @@
       </c>
       <c r="C25" s="1">
         <f t="shared" si="2"/>
-        <v>19000</v>
+        <v>8700</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.3">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="C26" s="1">
         <f t="shared" si="2"/>
-        <v>20500</v>
+        <v>9200</v>
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.3">
@@ -2182,7 +2182,7 @@
       </c>
       <c r="C27" s="1">
         <f t="shared" si="2"/>
-        <v>22000</v>
+        <v>9700</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.3">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="C28" s="1">
         <f t="shared" si="2"/>
-        <v>23500</v>
+        <v>10200</v>
       </c>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.3">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="C29" s="1">
         <f t="shared" si="2"/>
-        <v>25000</v>
+        <v>10700</v>
       </c>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.3">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="C30" s="1">
         <f t="shared" si="2"/>
-        <v>26500</v>
+        <v>11200</v>
       </c>
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.3">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="C31" s="1">
         <f t="shared" si="2"/>
-        <v>28000</v>
+        <v>11700</v>
       </c>
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.3">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="C32" s="1">
         <f t="shared" si="2"/>
-        <v>29500</v>
+        <v>12200</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.3">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="C33" s="1">
         <f>C32+$H$7</f>
-        <v>31500</v>
+        <v>12800</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.3">
@@ -2244,8 +2244,8 @@
         <v>32</v>
       </c>
       <c r="C34" s="1">
-        <f t="shared" ref="C34:C43" si="3">C33+$H$7</f>
-        <v>33500</v>
+        <f t="shared" ref="C34:C42" si="3">C33+$H$7</f>
+        <v>13400</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.3">
@@ -2254,7 +2254,7 @@
       </c>
       <c r="C35" s="1">
         <f t="shared" si="3"/>
-        <v>35500</v>
+        <v>14000</v>
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.3">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="C36" s="1">
         <f t="shared" si="3"/>
-        <v>37500</v>
+        <v>14600</v>
       </c>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.3">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="C37" s="1">
         <f t="shared" si="3"/>
-        <v>39500</v>
+        <v>15200</v>
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.3">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="C38" s="1">
         <f t="shared" si="3"/>
-        <v>41500</v>
+        <v>15800</v>
       </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.3">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="C39" s="1">
         <f t="shared" si="3"/>
-        <v>43500</v>
+        <v>16400</v>
       </c>
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.3">
@@ -2299,7 +2299,7 @@
       </c>
       <c r="C40" s="1">
         <f t="shared" si="3"/>
-        <v>45500</v>
+        <v>17000</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.3">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="C41" s="1">
         <f t="shared" si="3"/>
-        <v>47500</v>
+        <v>17600</v>
       </c>
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.3">
@@ -2317,7 +2317,7 @@
       </c>
       <c r="C42" s="1">
         <f t="shared" si="3"/>
-        <v>49500</v>
+        <v>18200</v>
       </c>
     </row>
     <row r="43" spans="2:3" x14ac:dyDescent="0.3">
@@ -2326,7 +2326,7 @@
       </c>
       <c r="C43" s="1">
         <f>C42+$H$8</f>
-        <v>52000</v>
+        <v>18900</v>
       </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.3">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="C44" s="1">
         <f t="shared" ref="C44:C52" si="4">C43+$H$8</f>
-        <v>54500</v>
+        <v>19600</v>
       </c>
     </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.3">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="C45" s="1">
         <f t="shared" si="4"/>
-        <v>57000</v>
+        <v>20300</v>
       </c>
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.3">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="C46" s="1">
         <f t="shared" si="4"/>
-        <v>59500</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.3">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="C47" s="1">
         <f t="shared" si="4"/>
-        <v>62000</v>
+        <v>21700</v>
       </c>
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.3">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="C48" s="1">
         <f t="shared" si="4"/>
-        <v>64500</v>
+        <v>22400</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.3">
@@ -2380,7 +2380,7 @@
       </c>
       <c r="C49" s="1">
         <f t="shared" si="4"/>
-        <v>67000</v>
+        <v>23100</v>
       </c>
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.3">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="C50" s="1">
         <f t="shared" si="4"/>
-        <v>69500</v>
+        <v>23800</v>
       </c>
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.3">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="C51" s="1">
         <f t="shared" si="4"/>
-        <v>72000</v>
+        <v>24500</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.3">
@@ -2407,7 +2407,7 @@
       </c>
       <c r="C52" s="1">
         <f t="shared" si="4"/>
-        <v>74500</v>
+        <v>25200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>